<commit_message>
renew varsList pubobsStation variables order
</commit_message>
<xml_diff>
--- a/data-raw/varsList.xlsx
+++ b/data-raw/varsList.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D04368A-74A3-4625-9051-14CA00A97054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A4FFF2-9EEE-4059-93EE-3343D179C9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7219" uniqueCount="1727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7231" uniqueCount="1728">
   <si>
     <t>variables</t>
   </si>
@@ -32782,6 +32782,10 @@
       </rPr>
       <t>类别</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年份</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -32789,7 +32793,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -32833,6 +32837,13 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <family val="1"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -32902,7 +32913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -32918,6 +32929,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -33214,7 +33226,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P617"/>
+  <dimension ref="A1:P618"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -58287,19 +58299,19 @@
     </row>
     <row r="588" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A588" s="1" t="str">
-        <f t="shared" ref="A588:A600" si="11">F588&amp;"_"&amp;G588&amp;"_"&amp;H588&amp;"_"&amp;I588</f>
-        <v>v99_obstation_list_index</v>
+        <f>F588&amp;"_"&amp;G588&amp;"_"&amp;H588&amp;"_"&amp;I588</f>
+        <v>v99_obstation_list_officer</v>
       </c>
       <c r="B588" s="1"/>
       <c r="C588" s="1" t="s">
-        <v>1707</v>
+        <v>1716</v>
       </c>
       <c r="D588" s="1" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="E588" s="1"/>
       <c r="F588" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="G588" s="1" t="s">
         <v>791</v>
@@ -58308,7 +58320,7 @@
         <v>785</v>
       </c>
       <c r="I588" s="1" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="J588" s="1" t="s">
         <v>1708</v>
@@ -58320,11 +58332,11 @@
         <v>1710</v>
       </c>
       <c r="M588" s="1" t="s">
-        <v>1707</v>
+        <v>1716</v>
       </c>
       <c r="N588" s="1"/>
       <c r="O588" s="1" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="P588" s="1" t="s">
         <v>1711</v>
@@ -58332,19 +58344,19 @@
     </row>
     <row r="589" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A589" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_name</v>
+        <f>F589&amp;"_"&amp;G589&amp;"_"&amp;H589&amp;"_"&amp;I589</f>
+        <v>v99_obstation_list_year</v>
       </c>
       <c r="B589" s="1"/>
-      <c r="C589" s="1" t="s">
-        <v>1712</v>
+      <c r="C589" s="7" t="s">
+        <v>1727</v>
       </c>
       <c r="D589" s="1" t="s">
-        <v>787</v>
+        <v>796</v>
       </c>
       <c r="E589" s="1"/>
       <c r="F589" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="G589" s="1" t="s">
         <v>791</v>
@@ -58353,7 +58365,7 @@
         <v>785</v>
       </c>
       <c r="I589" s="1" t="s">
-        <v>787</v>
+        <v>796</v>
       </c>
       <c r="J589" s="1" t="s">
         <v>1708</v>
@@ -58364,12 +58376,12 @@
       <c r="L589" s="1" t="s">
         <v>1710</v>
       </c>
-      <c r="M589" s="1" t="s">
-        <v>1713</v>
+      <c r="M589" s="7" t="s">
+        <v>1727</v>
       </c>
       <c r="N589" s="1"/>
       <c r="O589" s="1" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="P589" s="1" t="s">
         <v>1711</v>
@@ -58377,19 +58389,19 @@
     </row>
     <row r="590" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A590" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_institution</v>
+        <f t="shared" ref="A590:A601" si="11">F590&amp;"_"&amp;G590&amp;"_"&amp;H590&amp;"_"&amp;I590</f>
+        <v>v99_obstation_list_index</v>
       </c>
       <c r="B590" s="1"/>
       <c r="C590" s="1" t="s">
-        <v>1714</v>
+        <v>1707</v>
       </c>
       <c r="D590" s="1" t="s">
-        <v>699</v>
+        <v>786</v>
       </c>
       <c r="E590" s="1"/>
       <c r="F590" s="1" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="G590" s="1" t="s">
         <v>791</v>
@@ -58398,7 +58410,7 @@
         <v>785</v>
       </c>
       <c r="I590" s="1" t="s">
-        <v>699</v>
+        <v>786</v>
       </c>
       <c r="J590" s="1" t="s">
         <v>1708</v>
@@ -58410,11 +58422,11 @@
         <v>1710</v>
       </c>
       <c r="M590" s="1" t="s">
-        <v>1714</v>
+        <v>1707</v>
       </c>
       <c r="N590" s="1"/>
       <c r="O590" s="1" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="P590" s="1" t="s">
         <v>1711</v>
@@ -58423,18 +58435,18 @@
     <row r="591" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A591" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_obstation_list_administrator</v>
+        <v>v99_obstation_list_name</v>
       </c>
       <c r="B591" s="1"/>
       <c r="C591" s="1" t="s">
-        <v>1715</v>
+        <v>1712</v>
       </c>
       <c r="D591" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E591" s="1"/>
       <c r="F591" s="1" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="G591" s="1" t="s">
         <v>791</v>
@@ -58443,7 +58455,7 @@
         <v>785</v>
       </c>
       <c r="I591" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="J591" s="1" t="s">
         <v>1708</v>
@@ -58455,11 +58467,11 @@
         <v>1710</v>
       </c>
       <c r="M591" s="1" t="s">
-        <v>1715</v>
+        <v>1713</v>
       </c>
       <c r="N591" s="1"/>
       <c r="O591" s="1" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="P591" s="1" t="s">
         <v>1711</v>
@@ -58468,14 +58480,14 @@
     <row r="592" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A592" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_obstation_list_officer</v>
+        <v>v99_obstation_list_institution</v>
       </c>
       <c r="B592" s="1"/>
       <c r="C592" s="1" t="s">
-        <v>1716</v>
+        <v>1714</v>
       </c>
       <c r="D592" s="1" t="s">
-        <v>792</v>
+        <v>699</v>
       </c>
       <c r="E592" s="1"/>
       <c r="F592" s="1" t="s">
@@ -58488,7 +58500,7 @@
         <v>785</v>
       </c>
       <c r="I592" s="1" t="s">
-        <v>792</v>
+        <v>699</v>
       </c>
       <c r="J592" s="1" t="s">
         <v>1708</v>
@@ -58500,7 +58512,7 @@
         <v>1710</v>
       </c>
       <c r="M592" s="1" t="s">
-        <v>1716</v>
+        <v>1714</v>
       </c>
       <c r="N592" s="1"/>
       <c r="O592" s="1" t="s">
@@ -58513,14 +58525,14 @@
     <row r="593" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A593" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_obstation_list_province</v>
+        <v>v99_obstation_list_administrator</v>
       </c>
       <c r="B593" s="1"/>
       <c r="C593" s="1" t="s">
-        <v>1717</v>
+        <v>1715</v>
       </c>
       <c r="D593" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="E593" s="1"/>
       <c r="F593" s="1" t="s">
@@ -58533,7 +58545,7 @@
         <v>785</v>
       </c>
       <c r="I593" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="J593" s="1" t="s">
         <v>1708</v>
@@ -58545,7 +58557,7 @@
         <v>1710</v>
       </c>
       <c r="M593" s="1" t="s">
-        <v>1717</v>
+        <v>1715</v>
       </c>
       <c r="N593" s="1"/>
       <c r="O593" s="1" t="s">
@@ -58557,40 +58569,40 @@
     </row>
     <row r="594" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A594" s="1" t="str">
-        <f t="shared" ref="A594" si="12">F594&amp;"_"&amp;G594&amp;"_"&amp;H594&amp;"_"&amp;I594</f>
-        <v>v99_agripark_list_year</v>
+        <f t="shared" si="11"/>
+        <v>v99_obstation_list_province</v>
       </c>
       <c r="B594" s="1"/>
       <c r="C594" s="1" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="D594" s="1" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="E594" s="1"/>
       <c r="F594" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G594" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H594" s="1" t="s">
         <v>785</v>
       </c>
       <c r="I594" s="1" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="J594" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K594" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L594" s="1" t="s">
         <v>1710</v>
       </c>
       <c r="M594" s="1" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="N594" s="1"/>
       <c r="O594" s="1" t="s">
@@ -58602,15 +58614,15 @@
     </row>
     <row r="595" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A595" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_index</v>
+        <f t="shared" ref="A595" si="12">F595&amp;"_"&amp;G595&amp;"_"&amp;H595&amp;"_"&amp;I595</f>
+        <v>v99_agripark_list_year</v>
       </c>
       <c r="B595" s="1"/>
       <c r="C595" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="D595" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="E595" s="1"/>
       <c r="F595" s="1" t="s">
@@ -58623,7 +58635,7 @@
         <v>785</v>
       </c>
       <c r="I595" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="J595" s="1" t="s">
         <v>1708</v>
@@ -58635,7 +58647,7 @@
         <v>1710</v>
       </c>
       <c r="M595" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="N595" s="1"/>
       <c r="O595" s="1" t="s">
@@ -58648,14 +58660,14 @@
     <row r="596" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A596" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_agripark_list_batch</v>
+        <v>v99_agripark_list_index</v>
       </c>
       <c r="B596" s="1"/>
       <c r="C596" s="1" t="s">
-        <v>1720</v>
+        <v>1707</v>
       </c>
       <c r="D596" s="1" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="E596" s="1"/>
       <c r="F596" s="1" t="s">
@@ -58668,7 +58680,7 @@
         <v>785</v>
       </c>
       <c r="I596" s="1" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="J596" s="1" t="s">
         <v>1708</v>
@@ -58680,7 +58692,7 @@
         <v>1710</v>
       </c>
       <c r="M596" s="1" t="s">
-        <v>1720</v>
+        <v>1707</v>
       </c>
       <c r="N596" s="1"/>
       <c r="O596" s="1" t="s">
@@ -58693,14 +58705,14 @@
     <row r="597" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A597" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_agripark_list_name</v>
+        <v>v99_agripark_list_batch</v>
       </c>
       <c r="B597" s="1"/>
       <c r="C597" s="1" t="s">
-        <v>1712</v>
+        <v>1720</v>
       </c>
       <c r="D597" s="1" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="E597" s="1"/>
       <c r="F597" s="1" t="s">
@@ -58713,7 +58725,7 @@
         <v>785</v>
       </c>
       <c r="I597" s="1" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="J597" s="1" t="s">
         <v>1708</v>
@@ -58725,7 +58737,7 @@
         <v>1710</v>
       </c>
       <c r="M597" s="1" t="s">
-        <v>1712</v>
+        <v>1720</v>
       </c>
       <c r="N597" s="1"/>
       <c r="O597" s="1" t="s">
@@ -58738,14 +58750,14 @@
     <row r="598" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A598" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_agripark_list_province</v>
+        <v>v99_agripark_list_name</v>
       </c>
       <c r="B598" s="1"/>
       <c r="C598" s="1" t="s">
-        <v>1717</v>
+        <v>1712</v>
       </c>
       <c r="D598" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="E598" s="1"/>
       <c r="F598" s="1" t="s">
@@ -58758,7 +58770,7 @@
         <v>785</v>
       </c>
       <c r="I598" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="J598" s="1" t="s">
         <v>1708</v>
@@ -58770,7 +58782,7 @@
         <v>1710</v>
       </c>
       <c r="M598" s="1" t="s">
-        <v>1717</v>
+        <v>1712</v>
       </c>
       <c r="N598" s="1"/>
       <c r="O598" s="1" t="s">
@@ -58783,14 +58795,14 @@
     <row r="599" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A599" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_agripark_list_officer</v>
+        <v>v99_agripark_list_province</v>
       </c>
       <c r="B599" s="1"/>
       <c r="C599" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="D599" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="E599" s="1"/>
       <c r="F599" s="1" t="s">
@@ -58803,7 +58815,7 @@
         <v>785</v>
       </c>
       <c r="I599" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="J599" s="1" t="s">
         <v>1708</v>
@@ -58815,7 +58827,7 @@
         <v>1710</v>
       </c>
       <c r="M599" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="N599" s="1"/>
       <c r="O599" s="1" t="s">
@@ -58828,14 +58840,14 @@
     <row r="600" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A600" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>v99_agripark_eval_year</v>
+        <v>v99_agripark_list_officer</v>
       </c>
       <c r="B600" s="1"/>
       <c r="C600" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="D600" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="E600" s="1"/>
       <c r="F600" s="1" t="s">
@@ -58845,10 +58857,10 @@
         <v>793</v>
       </c>
       <c r="H600" s="1" t="s">
-        <v>797</v>
+        <v>785</v>
       </c>
       <c r="I600" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="J600" s="1" t="s">
         <v>1708</v>
@@ -58857,10 +58869,10 @@
         <v>1719</v>
       </c>
       <c r="L600" s="1" t="s">
-        <v>1721</v>
+        <v>1710</v>
       </c>
       <c r="M600" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="N600" s="1"/>
       <c r="O600" s="1" t="s">
@@ -58872,15 +58884,15 @@
     </row>
     <row r="601" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A601" s="1" t="str">
-        <f t="shared" ref="A601:A606" si="13">F601&amp;"_"&amp;G601&amp;"_"&amp;H601&amp;"_"&amp;I601</f>
-        <v>v99_agripark_eval_index</v>
+        <f t="shared" si="11"/>
+        <v>v99_agripark_eval_year</v>
       </c>
       <c r="B601" s="1"/>
       <c r="C601" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="D601" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="E601" s="1"/>
       <c r="F601" s="1" t="s">
@@ -58893,7 +58905,7 @@
         <v>797</v>
       </c>
       <c r="I601" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="J601" s="1" t="s">
         <v>1708</v>
@@ -58905,7 +58917,7 @@
         <v>1721</v>
       </c>
       <c r="M601" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="N601" s="1"/>
       <c r="O601" s="1" t="s">
@@ -58917,15 +58929,15 @@
     </row>
     <row r="602" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A602" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_eval_name</v>
+        <f t="shared" ref="A602:A607" si="13">F602&amp;"_"&amp;G602&amp;"_"&amp;H602&amp;"_"&amp;I602</f>
+        <v>v99_agripark_eval_index</v>
       </c>
       <c r="B602" s="1"/>
       <c r="C602" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="D602" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E602" s="1"/>
       <c r="F602" s="1" t="s">
@@ -58938,7 +58950,7 @@
         <v>797</v>
       </c>
       <c r="I602" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J602" s="1" t="s">
         <v>1708</v>
@@ -58950,7 +58962,7 @@
         <v>1721</v>
       </c>
       <c r="M602" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="N602" s="1"/>
       <c r="O602" s="1" t="s">
@@ -58962,8 +58974,8 @@
     </row>
     <row r="603" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A603" s="1" t="str">
-        <f t="shared" ref="A603" si="14">F603&amp;"_"&amp;G603&amp;"_"&amp;H603&amp;"_"&amp;I603</f>
-        <v>v99_agripark_eval_result</v>
+        <f t="shared" si="13"/>
+        <v>v99_agripark_eval_name</v>
       </c>
       <c r="B603" s="1"/>
       <c r="C603" s="1" t="s">
@@ -58983,7 +58995,7 @@
         <v>797</v>
       </c>
       <c r="I603" s="1" t="s">
-        <v>798</v>
+        <v>787</v>
       </c>
       <c r="J603" s="1" t="s">
         <v>1708</v>
@@ -58995,7 +59007,7 @@
         <v>1721</v>
       </c>
       <c r="M603" s="1" t="s">
-        <v>1722</v>
+        <v>1712</v>
       </c>
       <c r="N603" s="1"/>
       <c r="O603" s="1" t="s">
@@ -59007,15 +59019,15 @@
     </row>
     <row r="604" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A604" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_eval_province</v>
+        <f t="shared" ref="A604" si="14">F604&amp;"_"&amp;G604&amp;"_"&amp;H604&amp;"_"&amp;I604</f>
+        <v>v99_agripark_eval_result</v>
       </c>
       <c r="B604" s="1"/>
       <c r="C604" s="1" t="s">
-        <v>1717</v>
+        <v>1712</v>
       </c>
       <c r="D604" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="E604" s="1"/>
       <c r="F604" s="1" t="s">
@@ -59028,7 +59040,7 @@
         <v>797</v>
       </c>
       <c r="I604" s="1" t="s">
-        <v>789</v>
+        <v>798</v>
       </c>
       <c r="J604" s="1" t="s">
         <v>1708</v>
@@ -59040,7 +59052,7 @@
         <v>1721</v>
       </c>
       <c r="M604" s="1" t="s">
-        <v>1717</v>
+        <v>1722</v>
       </c>
       <c r="N604" s="1"/>
       <c r="O604" s="1" t="s">
@@ -59053,14 +59065,14 @@
     <row r="605" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A605" s="1" t="str">
         <f t="shared" si="13"/>
-        <v>v99_agripark_eval_officer</v>
+        <v>v99_agripark_eval_province</v>
       </c>
       <c r="B605" s="1"/>
       <c r="C605" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="D605" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="E605" s="1"/>
       <c r="F605" s="1" t="s">
@@ -59073,7 +59085,7 @@
         <v>797</v>
       </c>
       <c r="I605" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="J605" s="1" t="s">
         <v>1708</v>
@@ -59085,7 +59097,7 @@
         <v>1721</v>
       </c>
       <c r="M605" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="N605" s="1"/>
       <c r="O605" s="1" t="s">
@@ -59098,14 +59110,14 @@
     <row r="606" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A606" s="1" t="str">
         <f t="shared" si="13"/>
-        <v>v99_agripark_check_year</v>
+        <v>v99_agripark_eval_officer</v>
       </c>
       <c r="B606" s="1"/>
       <c r="C606" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="D606" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="E606" s="1"/>
       <c r="F606" s="1" t="s">
@@ -59115,10 +59127,10 @@
         <v>793</v>
       </c>
       <c r="H606" s="1" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="I606" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="J606" s="1" t="s">
         <v>1708</v>
@@ -59127,10 +59139,10 @@
         <v>1719</v>
       </c>
       <c r="L606" s="1" t="s">
-        <v>1723</v>
+        <v>1721</v>
       </c>
       <c r="M606" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="N606" s="1"/>
       <c r="O606" s="1" t="s">
@@ -59142,15 +59154,15 @@
     </row>
     <row r="607" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A607" s="1" t="str">
-        <f t="shared" ref="A607:A617" si="15">F607&amp;"_"&amp;G607&amp;"_"&amp;H607&amp;"_"&amp;I607</f>
-        <v>v99_agripark_check_index</v>
+        <f t="shared" si="13"/>
+        <v>v99_agripark_check_year</v>
       </c>
       <c r="B607" s="1"/>
       <c r="C607" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="D607" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="E607" s="1"/>
       <c r="F607" s="1" t="s">
@@ -59163,7 +59175,7 @@
         <v>799</v>
       </c>
       <c r="I607" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="J607" s="1" t="s">
         <v>1708</v>
@@ -59175,7 +59187,7 @@
         <v>1723</v>
       </c>
       <c r="M607" s="1" t="s">
-        <v>1707</v>
+        <v>1718</v>
       </c>
       <c r="N607" s="1"/>
       <c r="O607" s="1" t="s">
@@ -59187,15 +59199,15 @@
     </row>
     <row r="608" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A608" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agripark_check_name</v>
+        <f t="shared" ref="A608:A618" si="15">F608&amp;"_"&amp;G608&amp;"_"&amp;H608&amp;"_"&amp;I608</f>
+        <v>v99_agripark_check_index</v>
       </c>
       <c r="B608" s="1"/>
       <c r="C608" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="D608" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E608" s="1"/>
       <c r="F608" s="1" t="s">
@@ -59208,7 +59220,7 @@
         <v>799</v>
       </c>
       <c r="I608" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J608" s="1" t="s">
         <v>1708</v>
@@ -59220,7 +59232,7 @@
         <v>1723</v>
       </c>
       <c r="M608" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="N608" s="1"/>
       <c r="O608" s="1" t="s">
@@ -59233,7 +59245,7 @@
     <row r="609" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A609" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agripark_check_result</v>
+        <v>v99_agripark_check_name</v>
       </c>
       <c r="B609" s="1"/>
       <c r="C609" s="1" t="s">
@@ -59253,7 +59265,7 @@
         <v>799</v>
       </c>
       <c r="I609" s="1" t="s">
-        <v>798</v>
+        <v>787</v>
       </c>
       <c r="J609" s="1" t="s">
         <v>1708</v>
@@ -59265,7 +59277,7 @@
         <v>1723</v>
       </c>
       <c r="M609" s="1" t="s">
-        <v>1722</v>
+        <v>1712</v>
       </c>
       <c r="N609" s="1"/>
       <c r="O609" s="1" t="s">
@@ -59278,14 +59290,14 @@
     <row r="610" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A610" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agripark_check_province</v>
+        <v>v99_agripark_check_result</v>
       </c>
       <c r="B610" s="1"/>
       <c r="C610" s="1" t="s">
-        <v>1717</v>
+        <v>1712</v>
       </c>
       <c r="D610" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="E610" s="1"/>
       <c r="F610" s="1" t="s">
@@ -59298,7 +59310,7 @@
         <v>799</v>
       </c>
       <c r="I610" s="1" t="s">
-        <v>789</v>
+        <v>798</v>
       </c>
       <c r="J610" s="1" t="s">
         <v>1708</v>
@@ -59310,7 +59322,7 @@
         <v>1723</v>
       </c>
       <c r="M610" s="1" t="s">
-        <v>1717</v>
+        <v>1722</v>
       </c>
       <c r="N610" s="1"/>
       <c r="O610" s="1" t="s">
@@ -59323,14 +59335,14 @@
     <row r="611" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A611" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agripark_check_officer</v>
+        <v>v99_agripark_check_province</v>
       </c>
       <c r="B611" s="1"/>
       <c r="C611" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="D611" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="E611" s="1"/>
       <c r="F611" s="1" t="s">
@@ -59343,7 +59355,7 @@
         <v>799</v>
       </c>
       <c r="I611" s="1" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="J611" s="1" t="s">
         <v>1708</v>
@@ -59355,7 +59367,7 @@
         <v>1723</v>
       </c>
       <c r="M611" s="1" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="N611" s="1"/>
       <c r="O611" s="1" t="s">
@@ -59368,60 +59380,59 @@
     <row r="612" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A612" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_year</v>
+        <v>v99_agripark_check_officer</v>
       </c>
       <c r="B612" s="1"/>
       <c r="C612" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="D612" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="E612" s="1"/>
       <c r="F612" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G612" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H612" s="1" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="I612" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="J612" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K612" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L612" s="1" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="M612" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="N612" s="1"/>
       <c r="O612" s="1" t="s">
-        <v>803</v>
+        <v>794</v>
       </c>
       <c r="P612" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="613" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A613" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_batch</v>
+        <v>v99_agrimachine_county_year</v>
       </c>
       <c r="B613" s="1"/>
       <c r="C613" s="1" t="s">
-        <v>1720</v>
-      </c>
-      <c r="D613" s="1" t="str">
-        <f>I613</f>
-        <v>batch</v>
+        <v>1718</v>
+      </c>
+      <c r="D613" s="1" t="s">
+        <v>796</v>
       </c>
       <c r="E613" s="1"/>
       <c r="F613" s="1" t="s">
@@ -59434,7 +59445,7 @@
         <v>801</v>
       </c>
       <c r="I613" s="1" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="J613" s="1" t="s">
         <v>1708</v>
@@ -59446,7 +59457,7 @@
         <v>1724</v>
       </c>
       <c r="M613" s="1" t="s">
-        <v>1720</v>
+        <v>1718</v>
       </c>
       <c r="N613" s="1"/>
       <c r="O613" s="1" t="s">
@@ -59459,15 +59470,15 @@
     <row r="614" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A614" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_id</v>
+        <v>v99_agrimachine_county_batch</v>
       </c>
       <c r="B614" s="1"/>
       <c r="C614" s="1" t="s">
-        <v>1726</v>
+        <v>1720</v>
       </c>
       <c r="D614" s="1" t="str">
-        <f t="shared" ref="D614:D617" si="16">I614</f>
-        <v>id</v>
+        <f>I614</f>
+        <v>batch</v>
       </c>
       <c r="E614" s="1"/>
       <c r="F614" s="1" t="s">
@@ -59480,7 +59491,7 @@
         <v>801</v>
       </c>
       <c r="I614" s="1" t="s">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="J614" s="1" t="s">
         <v>1708</v>
@@ -59492,11 +59503,11 @@
         <v>1724</v>
       </c>
       <c r="M614" s="1" t="s">
-        <v>1726</v>
+        <v>1720</v>
       </c>
       <c r="N614" s="1"/>
       <c r="O614" s="1" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="P614" s="1" t="s">
         <v>1725</v>
@@ -59505,15 +59516,15 @@
     <row r="615" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A615" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_index</v>
+        <v>v99_agrimachine_county_id</v>
       </c>
       <c r="B615" s="1"/>
       <c r="C615" s="1" t="s">
-        <v>1707</v>
+        <v>1726</v>
       </c>
       <c r="D615" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>index</v>
+        <f t="shared" ref="D615:D618" si="16">I615</f>
+        <v>id</v>
       </c>
       <c r="E615" s="1"/>
       <c r="F615" s="1" t="s">
@@ -59526,7 +59537,7 @@
         <v>801</v>
       </c>
       <c r="I615" s="1" t="s">
-        <v>786</v>
+        <v>804</v>
       </c>
       <c r="J615" s="1" t="s">
         <v>1708</v>
@@ -59538,7 +59549,7 @@
         <v>1724</v>
       </c>
       <c r="M615" s="1" t="s">
-        <v>1707</v>
+        <v>1726</v>
       </c>
       <c r="N615" s="1"/>
       <c r="O615" s="1" t="s">
@@ -59551,15 +59562,15 @@
     <row r="616" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A616" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_province</v>
+        <v>v99_agrimachine_county_index</v>
       </c>
       <c r="B616" s="1"/>
       <c r="C616" s="1" t="s">
-        <v>1717</v>
+        <v>1707</v>
       </c>
       <c r="D616" s="1" t="str">
         <f t="shared" si="16"/>
-        <v>province</v>
+        <v>index</v>
       </c>
       <c r="E616" s="1"/>
       <c r="F616" s="1" t="s">
@@ -59572,7 +59583,7 @@
         <v>801</v>
       </c>
       <c r="I616" s="1" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="J616" s="1" t="s">
         <v>1708</v>
@@ -59584,7 +59595,7 @@
         <v>1724</v>
       </c>
       <c r="M616" s="1" t="s">
-        <v>1717</v>
+        <v>1707</v>
       </c>
       <c r="N616" s="1"/>
       <c r="O616" s="1" t="s">
@@ -59597,15 +59608,15 @@
     <row r="617" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A617" s="1" t="str">
         <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_name</v>
+        <v>v99_agrimachine_county_province</v>
       </c>
       <c r="B617" s="1"/>
       <c r="C617" s="1" t="s">
-        <v>1712</v>
+        <v>1717</v>
       </c>
       <c r="D617" s="1" t="str">
         <f t="shared" si="16"/>
-        <v>name</v>
+        <v>province</v>
       </c>
       <c r="E617" s="1"/>
       <c r="F617" s="1" t="s">
@@ -59618,7 +59629,7 @@
         <v>801</v>
       </c>
       <c r="I617" s="1" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="J617" s="1" t="s">
         <v>1708</v>
@@ -59630,13 +59641,59 @@
         <v>1724</v>
       </c>
       <c r="M617" s="1" t="s">
-        <v>1712</v>
+        <v>1717</v>
       </c>
       <c r="N617" s="1"/>
       <c r="O617" s="1" t="s">
         <v>802</v>
       </c>
       <c r="P617" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="618" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A618" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_name</v>
+      </c>
+      <c r="B618" s="1"/>
+      <c r="C618" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D618" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>name</v>
+      </c>
+      <c r="E618" s="1"/>
+      <c r="F618" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G618" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H618" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I618" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="J618" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K618" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L618" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M618" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N618" s="1"/>
+      <c r="O618" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="P618" s="1" t="s">
         <v>1725</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new dataset MachineService fly
</commit_message>
<xml_diff>
--- a/data-raw/varsList.xlsx
+++ b/data-raw/varsList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4EE0D3-0923-40F5-B6F7-ECE4C121C5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A60CDFF-ABEE-4081-BAB7-633F71307A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24533" yWindow="3270" windowWidth="24496" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-6885" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7442" uniqueCount="1762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7651" uniqueCount="1820">
   <si>
     <t>variables</t>
   </si>
@@ -33029,6 +33029,236 @@
   </si>
   <si>
     <t>授权</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fwzz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>rs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>zyhzs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>njh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>zjfw</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>njcyry</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>njwx</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农业机械化服务</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>服务组织和人员</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机化作业服务组织</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农业专业合作社</t>
+  </si>
+  <si>
+    <t>农机户</t>
+  </si>
+  <si>
+    <t>zyh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数C</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数D</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数E</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末机构数F</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数C</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数D</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数E</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数F</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年末人数G</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>中国农业机械工业年鉴</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农业机械化投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>czzj</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>kytr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tgtr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jbjs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jxgz</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>财政投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cztr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>建设投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>购置投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jstr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gztr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机户</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机化作业服务专业户</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机化中介服务组织</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>乡村农机从业人员</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机维修厂及维修点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>财政资金投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>科研投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>推广投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>基本建设投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农业机械购置投入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机服务效益</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>农机服务收入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>个</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>万元</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>zsr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>njfwsr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>服务总收入</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -33036,7 +33266,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -33094,6 +33324,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3B3B3B"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -33163,7 +33399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -33181,6 +33417,10 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -33477,7 +33717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P639"/>
+  <dimension ref="A1:P658"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -33487,9 +33727,9 @@
     <col min="5" max="5" width="7.85546875" customWidth="1"/>
     <col min="6" max="6" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" customWidth="1"/>
     <col min="13" max="13" width="20.42578125" customWidth="1"/>
     <col min="14" max="14" width="60.42578125" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="17.85546875" customWidth="1"/>
@@ -58103,7 +58343,7 @@
     </row>
     <row r="580" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A580" s="1" t="str">
-        <f t="shared" ref="A580:A608" si="8">F580&amp;"_"&amp;G580&amp;"_"&amp;H580&amp;"_"&amp;I580</f>
+        <f t="shared" ref="A580:A609" si="8">F580&amp;"_"&amp;G580&amp;"_"&amp;H580&amp;"_"&amp;I580</f>
         <v>v8_t7_cczcq_znc</v>
       </c>
       <c r="B580" s="1"/>
@@ -59350,895 +59590,803 @@
     </row>
     <row r="609" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A609" s="1" t="str">
-        <f>F609&amp;"_"&amp;G609&amp;"_"&amp;H609&amp;"_"&amp;I609</f>
-        <v>v99_obstation_list_officer</v>
+        <f t="shared" si="8"/>
+        <v>v9_t1_fwzz_jgs</v>
       </c>
       <c r="B609" s="1"/>
-      <c r="C609" s="1" t="s">
-        <v>1716</v>
-      </c>
-      <c r="D609" s="1" t="s">
-        <v>792</v>
-      </c>
-      <c r="E609" s="1"/>
+      <c r="C609" s="1"/>
+      <c r="D609" s="1"/>
+      <c r="E609" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F609" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G609" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H609" s="1" t="s">
-        <v>785</v>
+        <v>1763</v>
       </c>
       <c r="I609" s="1" t="s">
-        <v>792</v>
+        <v>554</v>
       </c>
       <c r="J609" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K609" s="1" t="s">
-        <v>1709</v>
+        <v>1771</v>
       </c>
       <c r="L609" s="1" t="s">
-        <v>1710</v>
-      </c>
-      <c r="M609" s="1" t="s">
-        <v>1716</v>
+        <v>1772</v>
+      </c>
+      <c r="M609" s="7" t="s">
+        <v>1776</v>
       </c>
       <c r="N609" s="1"/>
       <c r="O609" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P609" s="1" t="s">
-        <v>1711</v>
+        <v>1731</v>
+      </c>
+      <c r="P609" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="610" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A610" s="1" t="str">
-        <f>F610&amp;"_"&amp;G610&amp;"_"&amp;H610&amp;"_"&amp;I610</f>
-        <v>v99_obstation_list_year</v>
-      </c>
+      <c r="A610" s="1"/>
       <c r="B610" s="1"/>
-      <c r="C610" s="7" t="s">
-        <v>1727</v>
-      </c>
-      <c r="D610" s="1" t="s">
-        <v>796</v>
-      </c>
-      <c r="E610" s="1"/>
+      <c r="C610" s="1"/>
+      <c r="D610" s="1"/>
+      <c r="E610" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F610" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G610" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H610" s="1" t="s">
-        <v>785</v>
+        <v>1763</v>
       </c>
       <c r="I610" s="1" t="s">
-        <v>796</v>
+        <v>1764</v>
       </c>
       <c r="J610" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K610" s="1" t="s">
-        <v>1709</v>
+        <v>1771</v>
       </c>
       <c r="L610" s="1" t="s">
-        <v>1710</v>
+        <v>1772</v>
       </c>
       <c r="M610" s="7" t="s">
-        <v>1727</v>
+        <v>1782</v>
       </c>
       <c r="N610" s="1"/>
       <c r="O610" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P610" s="1" t="s">
-        <v>1711</v>
+        <v>1731</v>
+      </c>
+      <c r="P610" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="611" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A611" s="1" t="str">
-        <f t="shared" ref="A611:A622" si="11">F611&amp;"_"&amp;G611&amp;"_"&amp;H611&amp;"_"&amp;I611</f>
-        <v>v99_obstation_list_index</v>
-      </c>
+      <c r="A611" s="1"/>
       <c r="B611" s="1"/>
-      <c r="C611" s="1" t="s">
-        <v>1707</v>
-      </c>
-      <c r="D611" s="1" t="s">
-        <v>786</v>
-      </c>
-      <c r="E611" s="1"/>
+      <c r="C611" s="1"/>
+      <c r="D611" s="1"/>
+      <c r="E611" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F611" s="1" t="s">
-        <v>784</v>
+        <v>1762</v>
       </c>
       <c r="G611" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H611" s="1" t="s">
-        <v>785</v>
+        <v>1765</v>
       </c>
       <c r="I611" s="1" t="s">
-        <v>786</v>
+        <v>554</v>
       </c>
       <c r="J611" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K611" s="1" t="s">
-        <v>1709</v>
-      </c>
-      <c r="L611" s="1" t="s">
-        <v>1710</v>
-      </c>
-      <c r="M611" s="1" t="s">
-        <v>1707</v>
+        <v>1771</v>
+      </c>
+      <c r="L611" s="9" t="s">
+        <v>1773</v>
+      </c>
+      <c r="M611" s="7" t="s">
+        <v>1777</v>
       </c>
       <c r="N611" s="1"/>
       <c r="O611" s="1" t="s">
-        <v>790</v>
-      </c>
-      <c r="P611" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P611" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="612" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A612" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_name</v>
-      </c>
+      <c r="A612" s="1"/>
       <c r="B612" s="1"/>
-      <c r="C612" s="1" t="s">
-        <v>1712</v>
-      </c>
-      <c r="D612" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="E612" s="1"/>
+      <c r="C612" s="1"/>
+      <c r="D612" s="1"/>
+      <c r="E612" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F612" s="1" t="s">
-        <v>784</v>
+        <v>1762</v>
       </c>
       <c r="G612" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H612" s="1" t="s">
-        <v>785</v>
+        <v>1765</v>
       </c>
       <c r="I612" s="1" t="s">
-        <v>787</v>
+        <v>1764</v>
       </c>
       <c r="J612" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K612" s="1" t="s">
-        <v>1709</v>
-      </c>
-      <c r="L612" s="1" t="s">
-        <v>1710</v>
-      </c>
-      <c r="M612" s="1" t="s">
-        <v>1713</v>
+        <v>1771</v>
+      </c>
+      <c r="L612" s="9" t="s">
+        <v>1773</v>
+      </c>
+      <c r="M612" s="7" t="s">
+        <v>1783</v>
       </c>
       <c r="N612" s="1"/>
       <c r="O612" s="1" t="s">
-        <v>790</v>
-      </c>
-      <c r="P612" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P612" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="613" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A613" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_institution</v>
-      </c>
+      <c r="A613" s="1"/>
       <c r="B613" s="1"/>
-      <c r="C613" s="1" t="s">
-        <v>1714</v>
-      </c>
-      <c r="D613" s="1" t="s">
-        <v>699</v>
-      </c>
-      <c r="E613" s="1"/>
+      <c r="C613" s="1"/>
+      <c r="D613" s="1"/>
+      <c r="E613" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F613" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G613" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H613" s="1" t="s">
-        <v>785</v>
+        <v>1766</v>
       </c>
       <c r="I613" s="1" t="s">
-        <v>699</v>
+        <v>554</v>
       </c>
       <c r="J613" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K613" s="1" t="s">
-        <v>1709</v>
-      </c>
-      <c r="L613" s="1" t="s">
-        <v>1710</v>
-      </c>
-      <c r="M613" s="1" t="s">
-        <v>1714</v>
+        <v>1771</v>
+      </c>
+      <c r="L613" s="9" t="s">
+        <v>1774</v>
+      </c>
+      <c r="M613" s="7" t="s">
+        <v>1778</v>
       </c>
       <c r="N613" s="1"/>
       <c r="O613" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P613" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P613" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="614" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A614" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_administrator</v>
-      </c>
+      <c r="A614" s="1"/>
       <c r="B614" s="1"/>
-      <c r="C614" s="1" t="s">
-        <v>1715</v>
-      </c>
-      <c r="D614" s="1" t="s">
-        <v>788</v>
-      </c>
-      <c r="E614" s="1"/>
+      <c r="C614" s="1"/>
+      <c r="D614" s="1"/>
+      <c r="E614" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F614" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G614" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H614" s="1" t="s">
-        <v>785</v>
+        <v>1766</v>
       </c>
       <c r="I614" s="1" t="s">
-        <v>788</v>
+        <v>1764</v>
       </c>
       <c r="J614" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K614" s="1" t="s">
-        <v>1709</v>
+        <v>1771</v>
       </c>
       <c r="L614" s="1" t="s">
-        <v>1710</v>
+        <v>1802</v>
       </c>
       <c r="M614" s="1" t="s">
-        <v>1715</v>
+        <v>1784</v>
       </c>
       <c r="N614" s="1"/>
       <c r="O614" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P614" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P614" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="615" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A615" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_obstation_list_province</v>
-      </c>
+      <c r="A615" s="1"/>
       <c r="B615" s="1"/>
-      <c r="C615" s="1" t="s">
-        <v>1717</v>
-      </c>
-      <c r="D615" s="1" t="s">
-        <v>789</v>
-      </c>
-      <c r="E615" s="1"/>
+      <c r="C615" s="1"/>
+      <c r="D615" s="1"/>
+      <c r="E615" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F615" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G615" s="1" t="s">
-        <v>791</v>
+        <v>751</v>
       </c>
       <c r="H615" s="1" t="s">
-        <v>785</v>
+        <v>1775</v>
       </c>
       <c r="I615" s="1" t="s">
-        <v>789</v>
+        <v>554</v>
       </c>
       <c r="J615" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K615" s="1" t="s">
-        <v>1709</v>
+        <v>1771</v>
       </c>
       <c r="L615" s="1" t="s">
-        <v>1710</v>
+        <v>1803</v>
       </c>
       <c r="M615" s="1" t="s">
-        <v>1717</v>
+        <v>1779</v>
       </c>
       <c r="N615" s="1"/>
       <c r="O615" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P615" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P615" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="616" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A616" s="1" t="str">
-        <f t="shared" ref="A616" si="12">F616&amp;"_"&amp;G616&amp;"_"&amp;H616&amp;"_"&amp;I616</f>
-        <v>v99_agripark_list_year</v>
-      </c>
+      <c r="A616" s="1"/>
       <c r="B616" s="1"/>
-      <c r="C616" s="1" t="s">
-        <v>1718</v>
-      </c>
-      <c r="D616" s="1" t="s">
-        <v>796</v>
-      </c>
-      <c r="E616" s="1"/>
+      <c r="C616" s="1"/>
+      <c r="D616" s="1"/>
+      <c r="E616" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F616" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G616" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H616" s="1" t="s">
-        <v>785</v>
+        <v>1775</v>
       </c>
       <c r="I616" s="1" t="s">
-        <v>796</v>
+        <v>1764</v>
       </c>
       <c r="J616" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K616" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L616" s="1" t="s">
-        <v>1710</v>
+        <v>1803</v>
       </c>
       <c r="M616" s="1" t="s">
-        <v>1718</v>
+        <v>1785</v>
       </c>
       <c r="N616" s="1"/>
       <c r="O616" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P616" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P616" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="617" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A617" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_index</v>
-      </c>
+      <c r="A617" s="1"/>
       <c r="B617" s="1"/>
-      <c r="C617" s="1" t="s">
-        <v>1707</v>
-      </c>
-      <c r="D617" s="1" t="s">
-        <v>786</v>
-      </c>
-      <c r="E617" s="1"/>
+      <c r="C617" s="1"/>
+      <c r="D617" s="1"/>
+      <c r="E617" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F617" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G617" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H617" s="1" t="s">
-        <v>785</v>
+        <v>1767</v>
       </c>
       <c r="I617" s="1" t="s">
-        <v>786</v>
+        <v>554</v>
       </c>
       <c r="J617" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K617" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L617" s="1" t="s">
-        <v>1710</v>
+        <v>1804</v>
       </c>
       <c r="M617" s="1" t="s">
-        <v>1707</v>
+        <v>1780</v>
       </c>
       <c r="N617" s="1"/>
       <c r="O617" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P617" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P617" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="618" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A618" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_batch</v>
-      </c>
+      <c r="A618" s="1"/>
       <c r="B618" s="1"/>
-      <c r="C618" s="1" t="s">
-        <v>1720</v>
-      </c>
-      <c r="D618" s="1" t="s">
-        <v>795</v>
-      </c>
-      <c r="E618" s="1"/>
+      <c r="C618" s="1"/>
+      <c r="D618" s="1"/>
+      <c r="E618" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F618" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G618" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H618" s="1" t="s">
-        <v>785</v>
+        <v>1767</v>
       </c>
       <c r="I618" s="1" t="s">
-        <v>795</v>
+        <v>1764</v>
       </c>
       <c r="J618" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K618" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L618" s="1" t="s">
-        <v>1710</v>
+        <v>1804</v>
       </c>
       <c r="M618" s="1" t="s">
-        <v>1720</v>
+        <v>1786</v>
       </c>
       <c r="N618" s="1"/>
       <c r="O618" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P618" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P618" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="619" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A619" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_name</v>
-      </c>
+      <c r="A619" s="1"/>
       <c r="B619" s="1"/>
-      <c r="C619" s="1" t="s">
-        <v>1712</v>
-      </c>
-      <c r="D619" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="E619" s="1"/>
+      <c r="C619" s="1"/>
+      <c r="D619" s="1"/>
+      <c r="E619" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F619" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G619" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H619" s="1" t="s">
-        <v>785</v>
+        <v>1768</v>
       </c>
       <c r="I619" s="1" t="s">
-        <v>787</v>
+        <v>1764</v>
       </c>
       <c r="J619" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K619" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L619" s="1" t="s">
-        <v>1710</v>
+        <v>1805</v>
       </c>
       <c r="M619" s="1" t="s">
-        <v>1712</v>
+        <v>1788</v>
       </c>
       <c r="N619" s="1"/>
       <c r="O619" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P619" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P619" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="620" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A620" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_province</v>
-      </c>
+      <c r="A620" s="1"/>
       <c r="B620" s="1"/>
-      <c r="C620" s="1" t="s">
-        <v>1717</v>
-      </c>
-      <c r="D620" s="1" t="s">
-        <v>789</v>
-      </c>
-      <c r="E620" s="1"/>
+      <c r="C620" s="1"/>
+      <c r="D620" s="1"/>
+      <c r="E620" s="7" t="s">
+        <v>1814</v>
+      </c>
       <c r="F620" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G620" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H620" s="1" t="s">
-        <v>785</v>
+        <v>1769</v>
       </c>
       <c r="I620" s="1" t="s">
-        <v>789</v>
+        <v>554</v>
       </c>
       <c r="J620" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K620" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L620" s="1" t="s">
-        <v>1710</v>
+        <v>1806</v>
       </c>
       <c r="M620" s="1" t="s">
-        <v>1717</v>
+        <v>1781</v>
       </c>
       <c r="N620" s="1"/>
       <c r="O620" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P620" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P620" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="621" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A621" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_list_officer</v>
-      </c>
+      <c r="A621" s="1"/>
       <c r="B621" s="1"/>
-      <c r="C621" s="1" t="s">
-        <v>1716</v>
-      </c>
-      <c r="D621" s="1" t="s">
-        <v>792</v>
-      </c>
-      <c r="E621" s="1"/>
+      <c r="C621" s="1"/>
+      <c r="D621" s="1"/>
+      <c r="E621" s="7" t="s">
+        <v>1815</v>
+      </c>
       <c r="F621" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G621" s="1" t="s">
-        <v>793</v>
+        <v>751</v>
       </c>
       <c r="H621" s="1" t="s">
-        <v>785</v>
+        <v>1769</v>
       </c>
       <c r="I621" s="1" t="s">
-        <v>792</v>
+        <v>1764</v>
       </c>
       <c r="J621" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K621" s="1" t="s">
-        <v>1719</v>
+        <v>1771</v>
       </c>
       <c r="L621" s="1" t="s">
-        <v>1710</v>
+        <v>1806</v>
       </c>
       <c r="M621" s="1" t="s">
-        <v>1716</v>
+        <v>1787</v>
       </c>
       <c r="N621" s="1"/>
       <c r="O621" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P621" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P621" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="622" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A622" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>v99_agripark_eval_year</v>
-      </c>
+      <c r="A622" s="1"/>
       <c r="B622" s="1"/>
-      <c r="C622" s="1" t="s">
-        <v>1718</v>
-      </c>
-      <c r="D622" s="1" t="s">
-        <v>796</v>
-      </c>
-      <c r="E622" s="1"/>
+      <c r="C622" s="1"/>
+      <c r="D622" s="1"/>
+      <c r="E622" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F622" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G622" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H622" s="1" t="s">
-        <v>797</v>
+        <v>1797</v>
       </c>
       <c r="I622" s="1" t="s">
-        <v>796</v>
+        <v>1791</v>
       </c>
       <c r="J622" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K622" s="1" t="s">
-        <v>1719</v>
+        <v>1790</v>
       </c>
       <c r="L622" s="1" t="s">
-        <v>1721</v>
-      </c>
-      <c r="M622" s="1" t="s">
-        <v>1718</v>
+        <v>1796</v>
+      </c>
+      <c r="M622" s="10" t="s">
+        <v>1807</v>
       </c>
       <c r="N622" s="1"/>
       <c r="O622" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P622" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P622" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="623" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A623" s="1" t="str">
-        <f t="shared" ref="A623:A628" si="13">F623&amp;"_"&amp;G623&amp;"_"&amp;H623&amp;"_"&amp;I623</f>
-        <v>v99_agripark_eval_index</v>
-      </c>
+      <c r="A623" s="1"/>
       <c r="B623" s="1"/>
-      <c r="C623" s="1" t="s">
-        <v>1707</v>
-      </c>
-      <c r="D623" s="1" t="s">
-        <v>786</v>
-      </c>
-      <c r="E623" s="1"/>
+      <c r="C623" s="1"/>
+      <c r="D623" s="1"/>
+      <c r="E623" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F623" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G623" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H623" s="1" t="s">
-        <v>797</v>
+        <v>1797</v>
       </c>
       <c r="I623" s="1" t="s">
-        <v>786</v>
+        <v>1792</v>
       </c>
       <c r="J623" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K623" s="1" t="s">
-        <v>1719</v>
+        <v>1790</v>
       </c>
       <c r="L623" s="1" t="s">
-        <v>1721</v>
+        <v>1796</v>
       </c>
       <c r="M623" s="1" t="s">
-        <v>1707</v>
+        <v>1808</v>
       </c>
       <c r="N623" s="1"/>
       <c r="O623" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P623" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P623" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="624" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A624" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_eval_name</v>
-      </c>
+      <c r="A624" s="1"/>
       <c r="B624" s="1"/>
-      <c r="C624" s="1" t="s">
-        <v>1712</v>
-      </c>
-      <c r="D624" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="E624" s="1"/>
+      <c r="C624" s="1"/>
+      <c r="D624" s="1"/>
+      <c r="E624" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F624" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G624" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H624" s="1" t="s">
-        <v>797</v>
+        <v>1797</v>
       </c>
       <c r="I624" s="1" t="s">
-        <v>787</v>
+        <v>1793</v>
       </c>
       <c r="J624" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K624" s="1" t="s">
-        <v>1719</v>
+        <v>1790</v>
       </c>
       <c r="L624" s="1" t="s">
-        <v>1721</v>
+        <v>1796</v>
       </c>
       <c r="M624" s="1" t="s">
-        <v>1712</v>
+        <v>1809</v>
       </c>
       <c r="N624" s="1"/>
       <c r="O624" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P624" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P624" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="625" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A625" s="1" t="str">
-        <f t="shared" ref="A625" si="14">F625&amp;"_"&amp;G625&amp;"_"&amp;H625&amp;"_"&amp;I625</f>
-        <v>v99_agripark_eval_result</v>
-      </c>
+      <c r="A625" s="1"/>
       <c r="B625" s="1"/>
-      <c r="C625" s="1" t="s">
-        <v>1712</v>
-      </c>
-      <c r="D625" s="1" t="s">
-        <v>787</v>
-      </c>
-      <c r="E625" s="1"/>
+      <c r="C625" s="1"/>
+      <c r="D625" s="1"/>
+      <c r="E625" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F625" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G625" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H625" s="1" t="s">
-        <v>797</v>
+        <v>1800</v>
       </c>
       <c r="I625" s="1" t="s">
-        <v>798</v>
+        <v>1794</v>
       </c>
       <c r="J625" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K625" s="1" t="s">
-        <v>1719</v>
+        <v>1790</v>
       </c>
       <c r="L625" s="1" t="s">
-        <v>1721</v>
+        <v>1798</v>
       </c>
       <c r="M625" s="1" t="s">
-        <v>1722</v>
+        <v>1810</v>
       </c>
       <c r="N625" s="1"/>
       <c r="O625" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P625" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P625" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="626" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A626" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_eval_province</v>
-      </c>
+      <c r="A626" s="1"/>
       <c r="B626" s="1"/>
-      <c r="C626" s="1" t="s">
-        <v>1717</v>
-      </c>
-      <c r="D626" s="1" t="s">
-        <v>789</v>
-      </c>
-      <c r="E626" s="1"/>
+      <c r="C626" s="1"/>
+      <c r="D626" s="1"/>
+      <c r="E626" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F626" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G626" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H626" s="1" t="s">
-        <v>797</v>
+        <v>1801</v>
       </c>
       <c r="I626" s="1" t="s">
-        <v>789</v>
+        <v>1795</v>
       </c>
       <c r="J626" s="1" t="s">
-        <v>1708</v>
+        <v>1770</v>
       </c>
       <c r="K626" s="1" t="s">
-        <v>1719</v>
+        <v>1790</v>
       </c>
       <c r="L626" s="1" t="s">
-        <v>1721</v>
+        <v>1799</v>
       </c>
       <c r="M626" s="1" t="s">
-        <v>1717</v>
+        <v>1811</v>
       </c>
       <c r="N626" s="1"/>
       <c r="O626" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P626" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P626" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="627" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A627" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_eval_officer</v>
-      </c>
+      <c r="A627" s="1"/>
       <c r="B627" s="1"/>
-      <c r="C627" s="1" t="s">
-        <v>1716</v>
-      </c>
-      <c r="D627" s="1" t="s">
-        <v>792</v>
-      </c>
-      <c r="E627" s="1"/>
+      <c r="C627" s="1"/>
+      <c r="D627" s="1"/>
+      <c r="E627" s="7" t="s">
+        <v>1816</v>
+      </c>
       <c r="F627" s="1" t="s">
-        <v>783</v>
+        <v>1762</v>
       </c>
       <c r="G627" s="1" t="s">
-        <v>793</v>
+        <v>750</v>
       </c>
       <c r="H627" s="1" t="s">
-        <v>797</v>
+        <v>1817</v>
       </c>
       <c r="I627" s="1" t="s">
-        <v>792</v>
+        <v>1818</v>
       </c>
       <c r="J627" s="1" t="s">
-        <v>1708</v>
-      </c>
-      <c r="K627" s="1" t="s">
-        <v>1719</v>
-      </c>
-      <c r="L627" s="1" t="s">
-        <v>1721</v>
-      </c>
-      <c r="M627" s="1" t="s">
-        <v>1716</v>
+        <v>1770</v>
+      </c>
+      <c r="K627" s="10" t="s">
+        <v>1812</v>
+      </c>
+      <c r="L627" s="10" t="s">
+        <v>1819</v>
+      </c>
+      <c r="M627" s="10" t="s">
+        <v>1813</v>
       </c>
       <c r="N627" s="1"/>
       <c r="O627" s="1" t="s">
-        <v>794</v>
-      </c>
-      <c r="P627" s="1" t="s">
-        <v>1711</v>
+        <v>1738</v>
+      </c>
+      <c r="P627" s="7" t="s">
+        <v>1789</v>
       </c>
     </row>
     <row r="628" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A628" s="1" t="str">
-        <f t="shared" si="13"/>
-        <v>v99_agripark_check_year</v>
+        <f>F628&amp;"_"&amp;G628&amp;"_"&amp;H628&amp;"_"&amp;I628</f>
+        <v>v99_obstation_list_officer</v>
       </c>
       <c r="B628" s="1"/>
       <c r="C628" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="D628" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="E628" s="1"/>
       <c r="F628" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G628" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H628" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I628" s="1" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="J628" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K628" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L628" s="1" t="s">
-        <v>1723</v>
+        <v>1710</v>
       </c>
       <c r="M628" s="1" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
       <c r="N628" s="1"/>
       <c r="O628" s="1" t="s">
@@ -60250,40 +60398,40 @@
     </row>
     <row r="629" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A629" s="1" t="str">
-        <f t="shared" ref="A629:A639" si="15">F629&amp;"_"&amp;G629&amp;"_"&amp;H629&amp;"_"&amp;I629</f>
-        <v>v99_agripark_check_index</v>
+        <f>F629&amp;"_"&amp;G629&amp;"_"&amp;H629&amp;"_"&amp;I629</f>
+        <v>v99_obstation_list_year</v>
       </c>
       <c r="B629" s="1"/>
-      <c r="C629" s="1" t="s">
-        <v>1707</v>
+      <c r="C629" s="7" t="s">
+        <v>1727</v>
       </c>
       <c r="D629" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="E629" s="1"/>
       <c r="F629" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G629" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H629" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I629" s="1" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="J629" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K629" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L629" s="1" t="s">
-        <v>1723</v>
-      </c>
-      <c r="M629" s="1" t="s">
-        <v>1707</v>
+        <v>1710</v>
+      </c>
+      <c r="M629" s="7" t="s">
+        <v>1727</v>
       </c>
       <c r="N629" s="1"/>
       <c r="O629" s="1" t="s">
@@ -60295,44 +60443,44 @@
     </row>
     <row r="630" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A630" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agripark_check_name</v>
+        <f t="shared" ref="A630:A641" si="11">F630&amp;"_"&amp;G630&amp;"_"&amp;H630&amp;"_"&amp;I630</f>
+        <v>v99_obstation_list_index</v>
       </c>
       <c r="B630" s="1"/>
       <c r="C630" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="D630" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E630" s="1"/>
       <c r="F630" s="1" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="G630" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H630" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I630" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J630" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K630" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L630" s="1" t="s">
-        <v>1723</v>
+        <v>1710</v>
       </c>
       <c r="M630" s="1" t="s">
-        <v>1712</v>
+        <v>1707</v>
       </c>
       <c r="N630" s="1"/>
       <c r="O630" s="1" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="P630" s="1" t="s">
         <v>1711</v>
@@ -60340,8 +60488,8 @@
     </row>
     <row r="631" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A631" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agripark_check_result</v>
+        <f t="shared" si="11"/>
+        <v>v99_obstation_list_name</v>
       </c>
       <c r="B631" s="1"/>
       <c r="C631" s="1" t="s">
@@ -60352,32 +60500,32 @@
       </c>
       <c r="E631" s="1"/>
       <c r="F631" s="1" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="G631" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H631" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I631" s="1" t="s">
-        <v>798</v>
+        <v>787</v>
       </c>
       <c r="J631" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K631" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L631" s="1" t="s">
-        <v>1723</v>
+        <v>1710</v>
       </c>
       <c r="M631" s="1" t="s">
-        <v>1722</v>
+        <v>1713</v>
       </c>
       <c r="N631" s="1"/>
       <c r="O631" s="1" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="P631" s="1" t="s">
         <v>1711</v>
@@ -60385,40 +60533,40 @@
     </row>
     <row r="632" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A632" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agripark_check_province</v>
+        <f t="shared" si="11"/>
+        <v>v99_obstation_list_institution</v>
       </c>
       <c r="B632" s="1"/>
       <c r="C632" s="1" t="s">
-        <v>1717</v>
+        <v>1714</v>
       </c>
       <c r="D632" s="1" t="s">
-        <v>789</v>
+        <v>699</v>
       </c>
       <c r="E632" s="1"/>
       <c r="F632" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G632" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H632" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I632" s="1" t="s">
-        <v>789</v>
+        <v>699</v>
       </c>
       <c r="J632" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K632" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L632" s="1" t="s">
-        <v>1723</v>
+        <v>1710</v>
       </c>
       <c r="M632" s="1" t="s">
-        <v>1717</v>
+        <v>1714</v>
       </c>
       <c r="N632" s="1"/>
       <c r="O632" s="1" t="s">
@@ -60430,40 +60578,40 @@
     </row>
     <row r="633" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A633" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agripark_check_officer</v>
+        <f t="shared" si="11"/>
+        <v>v99_obstation_list_administrator</v>
       </c>
       <c r="B633" s="1"/>
       <c r="C633" s="1" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="D633" s="1" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="E633" s="1"/>
       <c r="F633" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G633" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H633" s="1" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="I633" s="1" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="J633" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K633" s="1" t="s">
-        <v>1719</v>
+        <v>1709</v>
       </c>
       <c r="L633" s="1" t="s">
-        <v>1723</v>
+        <v>1710</v>
       </c>
       <c r="M633" s="1" t="s">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="N633" s="1"/>
       <c r="O633" s="1" t="s">
@@ -60475,276 +60623,1131 @@
     </row>
     <row r="634" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A634" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_year</v>
+        <f t="shared" si="11"/>
+        <v>v99_obstation_list_province</v>
       </c>
       <c r="B634" s="1"/>
       <c r="C634" s="1" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="D634" s="1" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="E634" s="1"/>
       <c r="F634" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G634" s="1" t="s">
-        <v>800</v>
+        <v>791</v>
       </c>
       <c r="H634" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I634" s="1" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="J634" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K634" s="1" t="s">
-        <v>1611</v>
+        <v>1709</v>
       </c>
       <c r="L634" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M634" s="1" t="s">
-        <v>1718</v>
+        <v>1717</v>
       </c>
       <c r="N634" s="1"/>
       <c r="O634" s="1" t="s">
-        <v>803</v>
+        <v>794</v>
       </c>
       <c r="P634" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="635" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A635" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_batch</v>
+        <f t="shared" ref="A635" si="12">F635&amp;"_"&amp;G635&amp;"_"&amp;H635&amp;"_"&amp;I635</f>
+        <v>v99_agripark_list_year</v>
       </c>
       <c r="B635" s="1"/>
       <c r="C635" s="1" t="s">
-        <v>1720</v>
-      </c>
-      <c r="D635" s="1" t="str">
-        <f>I635</f>
-        <v>batch</v>
+        <v>1718</v>
+      </c>
+      <c r="D635" s="1" t="s">
+        <v>796</v>
       </c>
       <c r="E635" s="1"/>
       <c r="F635" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G635" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H635" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I635" s="1" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="J635" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K635" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L635" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M635" s="1" t="s">
-        <v>1720</v>
+        <v>1718</v>
       </c>
       <c r="N635" s="1"/>
       <c r="O635" s="1" t="s">
-        <v>803</v>
+        <v>794</v>
       </c>
       <c r="P635" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="636" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A636" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_id</v>
+        <f t="shared" si="11"/>
+        <v>v99_agripark_list_index</v>
       </c>
       <c r="B636" s="1"/>
       <c r="C636" s="1" t="s">
-        <v>1726</v>
-      </c>
-      <c r="D636" s="1" t="str">
-        <f t="shared" ref="D636:D639" si="16">I636</f>
-        <v>id</v>
+        <v>1707</v>
+      </c>
+      <c r="D636" s="1" t="s">
+        <v>786</v>
       </c>
       <c r="E636" s="1"/>
       <c r="F636" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G636" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H636" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I636" s="1" t="s">
-        <v>804</v>
+        <v>786</v>
       </c>
       <c r="J636" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K636" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L636" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M636" s="1" t="s">
-        <v>1726</v>
+        <v>1707</v>
       </c>
       <c r="N636" s="1"/>
       <c r="O636" s="1" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="P636" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="637" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A637" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_index</v>
+        <f t="shared" si="11"/>
+        <v>v99_agripark_list_batch</v>
       </c>
       <c r="B637" s="1"/>
       <c r="C637" s="1" t="s">
-        <v>1707</v>
-      </c>
-      <c r="D637" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>index</v>
+        <v>1720</v>
+      </c>
+      <c r="D637" s="1" t="s">
+        <v>795</v>
       </c>
       <c r="E637" s="1"/>
       <c r="F637" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G637" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H637" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I637" s="1" t="s">
-        <v>786</v>
+        <v>795</v>
       </c>
       <c r="J637" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K637" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L637" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M637" s="1" t="s">
-        <v>1707</v>
+        <v>1720</v>
       </c>
       <c r="N637" s="1"/>
       <c r="O637" s="1" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="P637" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="638" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A638" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_province</v>
+        <f t="shared" si="11"/>
+        <v>v99_agripark_list_name</v>
       </c>
       <c r="B638" s="1"/>
       <c r="C638" s="1" t="s">
-        <v>1717</v>
-      </c>
-      <c r="D638" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>province</v>
+        <v>1712</v>
+      </c>
+      <c r="D638" s="1" t="s">
+        <v>787</v>
       </c>
       <c r="E638" s="1"/>
       <c r="F638" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G638" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H638" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I638" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="J638" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K638" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L638" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M638" s="1" t="s">
-        <v>1717</v>
+        <v>1712</v>
       </c>
       <c r="N638" s="1"/>
       <c r="O638" s="1" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="P638" s="1" t="s">
-        <v>1725</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="639" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A639" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>v99_agrimachine_county_name</v>
+        <f t="shared" si="11"/>
+        <v>v99_agripark_list_province</v>
       </c>
       <c r="B639" s="1"/>
       <c r="C639" s="1" t="s">
-        <v>1712</v>
-      </c>
-      <c r="D639" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>name</v>
+        <v>1717</v>
+      </c>
+      <c r="D639" s="1" t="s">
+        <v>789</v>
       </c>
       <c r="E639" s="1"/>
       <c r="F639" s="1" t="s">
         <v>783</v>
       </c>
       <c r="G639" s="1" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="H639" s="1" t="s">
-        <v>801</v>
+        <v>785</v>
       </c>
       <c r="I639" s="1" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="J639" s="1" t="s">
         <v>1708</v>
       </c>
       <c r="K639" s="1" t="s">
-        <v>1611</v>
+        <v>1719</v>
       </c>
       <c r="L639" s="1" t="s">
-        <v>1724</v>
+        <v>1710</v>
       </c>
       <c r="M639" s="1" t="s">
-        <v>1712</v>
+        <v>1717</v>
       </c>
       <c r="N639" s="1"/>
       <c r="O639" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P639" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="640" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A640" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>v99_agripark_list_officer</v>
+      </c>
+      <c r="B640" s="1"/>
+      <c r="C640" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="D640" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="E640" s="1"/>
+      <c r="F640" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G640" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H640" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="I640" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="J640" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K640" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L640" s="1" t="s">
+        <v>1710</v>
+      </c>
+      <c r="M640" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="N640" s="1"/>
+      <c r="O640" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P640" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="641" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A641" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>v99_agripark_eval_year</v>
+      </c>
+      <c r="B641" s="1"/>
+      <c r="C641" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="D641" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="E641" s="1"/>
+      <c r="F641" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G641" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H641" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I641" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="J641" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K641" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L641" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M641" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="N641" s="1"/>
+      <c r="O641" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P641" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="642" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A642" s="1" t="str">
+        <f t="shared" ref="A642:A647" si="13">F642&amp;"_"&amp;G642&amp;"_"&amp;H642&amp;"_"&amp;I642</f>
+        <v>v99_agripark_eval_index</v>
+      </c>
+      <c r="B642" s="1"/>
+      <c r="C642" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="D642" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="E642" s="1"/>
+      <c r="F642" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G642" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H642" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I642" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="J642" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K642" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L642" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M642" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="N642" s="1"/>
+      <c r="O642" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P642" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="643" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A643" s="1" t="str">
+        <f t="shared" si="13"/>
+        <v>v99_agripark_eval_name</v>
+      </c>
+      <c r="B643" s="1"/>
+      <c r="C643" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D643" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="E643" s="1"/>
+      <c r="F643" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G643" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H643" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I643" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="J643" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K643" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L643" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M643" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N643" s="1"/>
+      <c r="O643" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P643" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="644" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A644" s="1" t="str">
+        <f t="shared" ref="A644" si="14">F644&amp;"_"&amp;G644&amp;"_"&amp;H644&amp;"_"&amp;I644</f>
+        <v>v99_agripark_eval_result</v>
+      </c>
+      <c r="B644" s="1"/>
+      <c r="C644" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D644" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="E644" s="1"/>
+      <c r="F644" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G644" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H644" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I644" s="1" t="s">
+        <v>798</v>
+      </c>
+      <c r="J644" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K644" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L644" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M644" s="1" t="s">
+        <v>1722</v>
+      </c>
+      <c r="N644" s="1"/>
+      <c r="O644" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P644" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="645" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A645" s="1" t="str">
+        <f t="shared" si="13"/>
+        <v>v99_agripark_eval_province</v>
+      </c>
+      <c r="B645" s="1"/>
+      <c r="C645" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D645" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="E645" s="1"/>
+      <c r="F645" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G645" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H645" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I645" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="J645" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K645" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L645" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M645" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="N645" s="1"/>
+      <c r="O645" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P645" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="646" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A646" s="1" t="str">
+        <f t="shared" si="13"/>
+        <v>v99_agripark_eval_officer</v>
+      </c>
+      <c r="B646" s="1"/>
+      <c r="C646" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="D646" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="E646" s="1"/>
+      <c r="F646" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G646" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H646" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="I646" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="J646" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K646" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L646" s="1" t="s">
+        <v>1721</v>
+      </c>
+      <c r="M646" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="N646" s="1"/>
+      <c r="O646" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P646" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="647" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A647" s="1" t="str">
+        <f t="shared" si="13"/>
+        <v>v99_agripark_check_year</v>
+      </c>
+      <c r="B647" s="1"/>
+      <c r="C647" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="D647" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="E647" s="1"/>
+      <c r="F647" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G647" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H647" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I647" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="J647" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K647" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L647" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M647" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="N647" s="1"/>
+      <c r="O647" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P647" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="648" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A648" s="1" t="str">
+        <f t="shared" ref="A648:A658" si="15">F648&amp;"_"&amp;G648&amp;"_"&amp;H648&amp;"_"&amp;I648</f>
+        <v>v99_agripark_check_index</v>
+      </c>
+      <c r="B648" s="1"/>
+      <c r="C648" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="D648" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="E648" s="1"/>
+      <c r="F648" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G648" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H648" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I648" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="J648" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K648" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L648" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M648" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="N648" s="1"/>
+      <c r="O648" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P648" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="649" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A649" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agripark_check_name</v>
+      </c>
+      <c r="B649" s="1"/>
+      <c r="C649" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D649" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="E649" s="1"/>
+      <c r="F649" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G649" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H649" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I649" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="J649" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K649" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L649" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M649" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N649" s="1"/>
+      <c r="O649" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P649" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="650" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A650" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agripark_check_result</v>
+      </c>
+      <c r="B650" s="1"/>
+      <c r="C650" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D650" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="E650" s="1"/>
+      <c r="F650" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G650" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H650" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I650" s="1" t="s">
+        <v>798</v>
+      </c>
+      <c r="J650" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K650" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L650" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M650" s="1" t="s">
+        <v>1722</v>
+      </c>
+      <c r="N650" s="1"/>
+      <c r="O650" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P650" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="651" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A651" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agripark_check_province</v>
+      </c>
+      <c r="B651" s="1"/>
+      <c r="C651" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D651" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="E651" s="1"/>
+      <c r="F651" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G651" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H651" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I651" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="J651" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K651" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L651" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M651" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="N651" s="1"/>
+      <c r="O651" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P651" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="652" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A652" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agripark_check_officer</v>
+      </c>
+      <c r="B652" s="1"/>
+      <c r="C652" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="D652" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="E652" s="1"/>
+      <c r="F652" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G652" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H652" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="I652" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="J652" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K652" s="1" t="s">
+        <v>1719</v>
+      </c>
+      <c r="L652" s="1" t="s">
+        <v>1723</v>
+      </c>
+      <c r="M652" s="1" t="s">
+        <v>1716</v>
+      </c>
+      <c r="N652" s="1"/>
+      <c r="O652" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="P652" s="1" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="653" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A653" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_year</v>
+      </c>
+      <c r="B653" s="1"/>
+      <c r="C653" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="D653" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="E653" s="1"/>
+      <c r="F653" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G653" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H653" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I653" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="J653" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K653" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L653" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M653" s="1" t="s">
+        <v>1718</v>
+      </c>
+      <c r="N653" s="1"/>
+      <c r="O653" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="P653" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="654" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A654" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_batch</v>
+      </c>
+      <c r="B654" s="1"/>
+      <c r="C654" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="D654" s="1" t="str">
+        <f>I654</f>
+        <v>batch</v>
+      </c>
+      <c r="E654" s="1"/>
+      <c r="F654" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G654" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H654" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I654" s="1" t="s">
+        <v>795</v>
+      </c>
+      <c r="J654" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K654" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L654" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M654" s="1" t="s">
+        <v>1720</v>
+      </c>
+      <c r="N654" s="1"/>
+      <c r="O654" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="P654" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="655" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A655" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_id</v>
+      </c>
+      <c r="B655" s="1"/>
+      <c r="C655" s="1" t="s">
+        <v>1726</v>
+      </c>
+      <c r="D655" s="1" t="str">
+        <f t="shared" ref="D655:D658" si="16">I655</f>
+        <v>id</v>
+      </c>
+      <c r="E655" s="1"/>
+      <c r="F655" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G655" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H655" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I655" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="J655" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K655" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L655" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M655" s="1" t="s">
+        <v>1726</v>
+      </c>
+      <c r="N655" s="1"/>
+      <c r="O655" s="1" t="s">
         <v>802</v>
       </c>
-      <c r="P639" s="1" t="s">
+      <c r="P655" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="656" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A656" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_index</v>
+      </c>
+      <c r="B656" s="1"/>
+      <c r="C656" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="D656" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>index</v>
+      </c>
+      <c r="E656" s="1"/>
+      <c r="F656" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G656" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H656" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I656" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="J656" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K656" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L656" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M656" s="1" t="s">
+        <v>1707</v>
+      </c>
+      <c r="N656" s="1"/>
+      <c r="O656" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="P656" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="657" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A657" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_province</v>
+      </c>
+      <c r="B657" s="1"/>
+      <c r="C657" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D657" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>province</v>
+      </c>
+      <c r="E657" s="1"/>
+      <c r="F657" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G657" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H657" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I657" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="J657" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K657" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L657" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M657" s="1" t="s">
+        <v>1717</v>
+      </c>
+      <c r="N657" s="1"/>
+      <c r="O657" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="P657" s="1" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="658" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A658" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>v99_agrimachine_county_name</v>
+      </c>
+      <c r="B658" s="1"/>
+      <c r="C658" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D658" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>name</v>
+      </c>
+      <c r="E658" s="1"/>
+      <c r="F658" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="G658" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="H658" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="I658" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="J658" s="1" t="s">
+        <v>1708</v>
+      </c>
+      <c r="K658" s="1" t="s">
+        <v>1611</v>
+      </c>
+      <c r="L658" s="1" t="s">
+        <v>1724</v>
+      </c>
+      <c r="M658" s="1" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N658" s="1"/>
+      <c r="O658" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="P658" s="1" t="s">
         <v>1725</v>
       </c>
     </row>

</xml_diff>